<commit_message>
refactor: Game networker 추가 및 리팩토링. data: Inventory 초기 세팅 데이타 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/ItemTable.xlsx
+++ b/input/Domains/Game/ItemTable.xlsx
@@ -1,35 +1,113 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31160598-292C-B84C-8B83-1FC804D359A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="1380" yWindow="500" windowWidth="37020" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="EQUIP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CARD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EQUIP" sheetId="1" r:id="rId1"/>
+    <sheet name="CARD" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+  <si>
+    <t>equipId</t>
+  </si>
+  <si>
+    <t>nameId</t>
+  </si>
+  <si>
+    <t>descId</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>pk</t>
+  </si>
+  <si>
+    <t>장비 ID (정본)</t>
+  </si>
+  <si>
+    <t>이름 텍스트 ID</t>
+  </si>
+  <si>
+    <t>설명 텍스트 ID</t>
+  </si>
+  <si>
+    <t>cardId</t>
+  </si>
+  <si>
+    <t>카드 ID (정본)</t>
+  </si>
+  <si>
+    <t>equip_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>equip_002</t>
+  </si>
+  <si>
+    <t>equip_003</t>
+  </si>
+  <si>
+    <t>equip_004</t>
+  </si>
+  <si>
+    <t>equip_005</t>
+  </si>
+  <si>
+    <t>card_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>card_002</t>
+  </si>
+  <si>
+    <t>card_003</t>
+  </si>
+  <si>
+    <t>card_004</t>
+  </si>
+  <si>
+    <t>card_005</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2">
     <font>
-      <name val="Calibri"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -48,80 +126,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -409,145 +428,152 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>equipId</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>nameId</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>descId</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>pk</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>장비 ID (정본)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>이름 텍스트 ID</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>설명 텍스트 ID</t>
-        </is>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>cardId</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>nameId</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>descId</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>pk</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>카드 ID (정본)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>이름 텍스트 ID</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>설명 텍스트 ID</t>
-        </is>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feature: item level 테이블 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/ItemTable.xlsx
+++ b/input/Domains/Game/ItemTable.xlsx
@@ -8,25 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388198F4-D2D7-504A-9CF9-BF2904867544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A5F9A42-8A81-B341-9065-2C4E2F806766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="1560" windowWidth="29240" windowHeight="17860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="41060" yWindow="-700" windowWidth="29240" windowHeight="17860" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ITEM_HERO" sheetId="7" r:id="rId1"/>
-    <sheet name="ITEM_EQUIP" sheetId="1" r:id="rId2"/>
-    <sheet name="ITEM_CARD" sheetId="2" r:id="rId3"/>
-    <sheet name="ITEM_MATERIAL" sheetId="6" r:id="rId4"/>
-    <sheet name="ITEM_TREASURE" sheetId="3" r:id="rId5"/>
-    <sheet name="ITEM_RENTAL" sheetId="4" r:id="rId6"/>
-    <sheet name="ITEM_PASS" sheetId="5" r:id="rId7"/>
+    <sheet name="ITEM_HERO_LEVEL" sheetId="9" r:id="rId2"/>
+    <sheet name="ITEM_EQUIP" sheetId="1" r:id="rId3"/>
+    <sheet name="ITEM_EQUIP_LEVEL" sheetId="10" r:id="rId4"/>
+    <sheet name="ITEM_CARD" sheetId="2" r:id="rId5"/>
+    <sheet name="ITEM_CARD_LEVEL" sheetId="11" r:id="rId6"/>
+    <sheet name="ITEM_MATERIAL" sheetId="6" r:id="rId7"/>
+    <sheet name="ITEM_RENTAL" sheetId="4" r:id="rId8"/>
+    <sheet name="ITEM_PASS" sheetId="5" r:id="rId9"/>
+    <sheet name="ITEM_TREASURE" sheetId="3" r:id="rId10"/>
+    <sheet name="REWARD@TREASURE" sheetId="8" r:id="rId11"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="60">
   <si>
     <t>nameId</t>
   </si>
@@ -49,39 +53,9 @@
     <t>설명 텍스트 ID</t>
   </si>
   <si>
-    <t>equip_001</t>
-  </si>
-  <si>
-    <t>equip_002</t>
-  </si>
-  <si>
-    <t>equip_003</t>
-  </si>
-  <si>
-    <t>equip_004</t>
-  </si>
-  <si>
-    <t>equip_005</t>
-  </si>
-  <si>
     <t>카드 ID (정본)</t>
   </si>
   <si>
-    <t>card_001</t>
-  </si>
-  <si>
-    <t>card_002</t>
-  </si>
-  <si>
-    <t>card_003</t>
-  </si>
-  <si>
-    <t>card_004</t>
-  </si>
-  <si>
-    <t>card_005</t>
-  </si>
-  <si>
     <t>chestNum</t>
   </si>
   <si>
@@ -94,15 +68,6 @@
     <t>상자 ID</t>
   </si>
   <si>
-    <t>chest_001</t>
-  </si>
-  <si>
-    <t>reward_chest_001_01</t>
-  </si>
-  <si>
-    <t>reward_chest_001_02</t>
-  </si>
-  <si>
     <t>NO_ADS</t>
   </si>
   <si>
@@ -122,23 +87,147 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>유닛 ID (정본)</t>
-  </si>
-  <si>
-    <t>hero_001</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>hero_002</t>
-  </si>
-  <si>
-    <t>hero_003</t>
-  </si>
-  <si>
-    <t>hero_004</t>
-  </si>
-  <si>
-    <t>hero_005</t>
+    <t>reward_treasure_001_01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reward_treasure_001_02</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>rewardNum</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>rate</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>enum:REWARD_TYPE</t>
+  </si>
+  <si>
+    <t>float</t>
+  </si>
+  <si>
+    <t>Reward PK (auto-increment number)</t>
+  </si>
+  <si>
+    <t>Reward Group Key</t>
+  </si>
+  <si>
+    <t>Reward Type</t>
+  </si>
+  <si>
+    <t>Target ID</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>CURRENCY</t>
+  </si>
+  <si>
+    <t>JEWEL_FREE</t>
+  </si>
+  <si>
+    <t>item_treasure_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>item_card_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>item_equip_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>item_hero_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>group:true</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>unitId</t>
+  </si>
+  <si>
+    <t>unit_hero_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>유닛 ID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>아이템 ID (정본)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>int</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>itemLevel</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>item_hero_001</t>
+  </si>
+  <si>
+    <t>item_equip_001</t>
+  </si>
+  <si>
+    <t>item_card_001</t>
+  </si>
+  <si>
+    <t>STAT_TYPE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>statType00</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>statValue01</t>
+  </si>
+  <si>
+    <t>statValue00</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>statType01</t>
+  </si>
+  <si>
+    <t>statType02</t>
+  </si>
+  <si>
+    <t>statValue02</t>
+  </si>
+  <si>
+    <t>statType03</t>
+  </si>
+  <si>
+    <t>statValue03</t>
+  </si>
+  <si>
+    <t>UNIT_HP_MAX</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>index</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -485,73 +574,265 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA853EB1-71B0-5C41-BB38-1A705283C6EA}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
-    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
+  <cols>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="18.6640625" customWidth="1"/>
+    <col min="4" max="4" width="23.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEA2C6C1-4D13-EB4F-906F-FDD52B5821C1}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
+  <cols>
+    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
         <v>30</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
+      <c r="D5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>36</v>
+      <c r="E5">
+        <v>1000</v>
+      </c>
+      <c r="F5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6">
+        <v>100</v>
+      </c>
+      <c r="F6">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -561,8 +842,191 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0C9BDCD-CAFF-D048-871C-88596981A0D3}">
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
+  <cols>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="B4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9">
+        <v>140</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
@@ -570,7 +1034,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -608,101 +1072,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -712,35 +1082,149 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91CB880A-6343-1D47-A4BA-B1C5531C394D}">
-  <dimension ref="A1:C3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD3681BF-21FC-F74E-B81F-6FDC4E483296}">
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
+  <cols>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="B4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>3</v>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -750,75 +1234,206 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <cols>
+    <col min="1" max="1" width="22.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF92740-2D83-6444-936A-7C5DEEEB21BB}">
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="18.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="D1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+        <v>50</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>44</v>
+      </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="D2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>49</v>
+      </c>
+      <c r="E2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>36</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6">
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" t="s">
-        <v>24</v>
+        <v>36</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -827,7 +1442,45 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91CB880A-6343-1D47-A4BA-B1C5531C394D}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
@@ -837,7 +1490,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -863,7 +1516,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -872,7 +1525,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
@@ -882,7 +1535,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -917,22 +1570,22 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feature: item equip 장착 로직 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/ItemTable.xlsx
+++ b/input/Domains/Game/ItemTable.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="41060" yWindow="-700" windowWidth="29240" windowHeight="17860" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_HERO" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_HERO_LEVEL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_EQUIP" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_EQUIP_LEVEL" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_CARD" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_CARD_LEVEL" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_MATERIAL" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_RENTAL" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_PASS" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_TREASURE" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REWARD@TREASURE" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="ITEM_HERO" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ITEM_HERO_LEVEL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ITEM_EQUIP" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ITEM_EQUIP_LEVEL" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ITEM_CARD" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ITEM_CARD_LEVEL" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ITEM_MATERIAL" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ITEM_RENTAL" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ITEM_PASS" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ITEM_TREASURE" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="REWARD@TREASURE" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1073,7 +1073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="14.83203125" customWidth="1" min="1" max="1"/>
@@ -1095,6 +1095,11 @@
           <t>desc_id</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>equip_type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1112,6 +1117,11 @@
           <t>string</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>enum:EQUIP_TYPE</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1136,11 +1146,21 @@
           <t>설명 텍스트 ID</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>장비 타입 (EQUIP_SLOT 규칙 키)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
           <t>item_equip_001</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SWORD</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: contract json 파일 정리.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/ItemTable.xlsx
+++ b/input/Domains/Game/ItemTable.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="41060" yWindow="-700" windowWidth="29240" windowHeight="17860" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4180" yWindow="1600" windowWidth="29240" windowHeight="17860" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ITEM_HERO" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ITEM_HERO_LEVEL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ITEM_EQUIP" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ITEM_EQUIP_LEVEL" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ITEM_CARD" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ITEM_CARD_LEVEL" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ITEM_MATERIAL" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ITEM_RENTAL" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ITEM_PASS" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="ITEM_TREASURE" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="REWARD@TREASURE" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_HERO" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_HERO_LEVEL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUIP_SLOT" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_EQUIP" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_EQUIP_LEVEL" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_CARD" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_CARD_LEVEL" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_MATERIAL" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_RENTAL" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_PASS" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEM_TREASURE" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REWARD@TREASURE" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -532,6 +533,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
+  <cols>
+    <col width="13.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>item_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>desc_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>pk</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>이름 텍스트 ID</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>설명 텍스트 ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P2026_01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P2026_02</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P2026_03</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P2026_04</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
@@ -638,7 +737,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -899,7 +998,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>STAT_TYPE</t>
+          <t>UNIT_STAT_TYPE</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -909,7 +1008,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>STAT_TYPE</t>
+          <t>UNIT_STAT_TYPE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -919,7 +1018,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>STAT_TYPE</t>
+          <t>UNIT_STAT_TYPE</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -929,7 +1028,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>STAT_TYPE</t>
+          <t>UNIT_STAT_TYPE</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1073,59 +1172,219 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
-    <col width="14.83203125" customWidth="1" min="1" max="1"/>
+    <col width="19.5" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="23.5" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="22.1640625" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>item_id</t>
+          <t>equip_type</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>name_id</t>
+          <t>allowed_slots</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>desc_id</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>equip_type</t>
+          <t>two_handed</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum:EQUIP_TYPE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>EQUIP_SLOT_TYPE[]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>enum:EQUIP_TYPE</t>
+          <t>bool</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>pk, gen:EQUIP_TYPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>착용 가능한 slot</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Off Hand 를 비워야 함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SWORD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HAND_MAIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BOW</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HAND_MAIN</t>
+        </is>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SHIELD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HAND_SUB</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HELMET</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GLOVES</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GLOVES</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RING</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RING_LEFT, RING_RIGHT</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <cols>
+    <col width="22.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22.33203125" bestFit="1" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>item_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>desc_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>equip_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>upgrade_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>enum:EQUIP_TYPE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>pk</t>
         </is>
       </c>
@@ -1155,10 +1414,44 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>item_equip_001</t>
+          <t>item_equip_sword_001</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
+        <is>
+          <t>SWORD</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>item_equip_sword_002</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>item_equip_sword_002</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SWORD</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>item_equip_sword_003</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>item_equip_sword_003</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>SWORD</t>
         </is>
@@ -1169,7 +1462,434 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
+  <cols>
+    <col width="22.33203125" bestFit="1" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>item_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>item_level</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>stat_type00</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>stat_value00</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>stat_type01</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>stat_value01</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>stat_type02</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>stat_value02</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>stat_type03</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>stat_value03</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>UNIT_STAT_TYPE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>UNIT_STAT_TYPE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>UNIT_STAT_TYPE</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UNIT_STAT_TYPE</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>pk</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>group:true</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>아이템 ID (정본)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>item_equip_sword_001</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>item_equip_sword_001</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>item_equip_sword_001</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>item_equip_sword_001</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>item_equip_sword_001</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>item_equip_sword_002</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>item_equip_sword_002</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>item_equip_sword_002</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>item_equip_sword_002</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>item_equip_sword_002</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>item_equip_sword_003</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>item_equip_sword_003</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>item_equip_sword_003</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>item_equip_sword_003</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>item_equip_sword_003</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <cols>
+    <col width="22.1640625" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>item_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>desc_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>pk</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>카드 ID (정본)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>이름 텍스트 ID</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>설명 텍스트 ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>item_card_001</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1256,7 +1976,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>STAT_TYPE</t>
+          <t>UNIT_STAT_TYPE</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1266,7 +1986,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>STAT_TYPE</t>
+          <t>UNIT_STAT_TYPE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1276,7 +1996,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>STAT_TYPE</t>
+          <t>UNIT_STAT_TYPE</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1286,7 +2006,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>STAT_TYPE</t>
+          <t>UNIT_STAT_TYPE</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1320,7 +2040,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>item_equip_001</t>
+          <t>item_card_001</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1333,7 +2053,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>item_equip_001</t>
+          <t>item_card_001</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1346,7 +2066,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>item_equip_001</t>
+          <t>item_card_001</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1359,7 +2079,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>item_equip_001</t>
+          <t>item_card_001</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1372,7 +2092,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>item_equip_001</t>
+          <t>item_card_001</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1384,304 +2104,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
-  <cols>
-    <col width="22.1640625" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>item_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>name_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>desc_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>pk</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>카드 ID (정본)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>이름 텍스트 ID</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>설명 텍스트 ID</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>item_card_001</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
-  <cols>
-    <col width="15.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>index</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>item_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>item_level</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>stat_type00</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>stat_value00</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>stat_type01</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>stat_value01</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>stat_type02</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>stat_value02</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>stat_type03</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>stat_value03</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>STAT_TYPE</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>STAT_TYPE</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>STAT_TYPE</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>STAT_TYPE</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>pk</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>group:true</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>아이템 ID (정본)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>item_card_001</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>item_card_001</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>item_card_001</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>item_card_001</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>item_card_001</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1736,7 +2159,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1796,102 +2219,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
-  <cols>
-    <col width="13.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>item_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>name_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>desc_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>pk</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>이름 텍스트 ID</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>설명 텍스트 ID</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>P2026_01</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>P2026_02</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>P2026_03</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>P2026_04</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>